<commit_message>
corrected new time entry with the 'name'
</commit_message>
<xml_diff>
--- a/data/Pajjota.xlsx
+++ b/data/Pajjota.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -97,7 +97,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -118,11 +118,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -167,7 +162,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -177,10 +172,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -204,37 +195,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -310,7 +301,7 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.37"/>
   </cols>
   <sheetData>
@@ -355,10 +346,10 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -446,8 +437,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.75"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
@@ -459,6 +453,11 @@
       <c r="C1" s="2" t="s">
         <v>21</v>
       </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
fill dhamma.org gaps with 'fillin' period
</commit_message>
<xml_diff>
--- a/data/Pajjota.xlsx
+++ b/data/Pajjota.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t xml:space="preserve">container</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fillin</t>
   </si>
 </sst>
 </file>
@@ -475,8 +478,12 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="C2" s="2"/>
     </row>
   </sheetData>

</xml_diff>